<commit_message>
Sync all Excel downloads (EXCEL/ 1-9 + golden) to current platform data - page 7 = 34 rows
</commit_message>
<xml_diff>
--- a/EXCEL/1 - DASHBOARD.xlsx
+++ b/EXCEL/1 - DASHBOARD.xlsx
@@ -1144,30 +1144,30 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="n">
-        <v>23533</v>
+        <v>23532</v>
       </c>
       <c r="B2" s="9" t="n">
-        <v>8810</v>
+        <v>8963</v>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="D2" s="11" t="n">
-        <v>2724</v>
+        <v>2751</v>
       </c>
       <c r="E2" s="9" t="n">
         <v>521</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>2203</v>
+        <v>2230</v>
       </c>
       <c r="G2" s="8" t="n">
         <v>290</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
@@ -1348,7 +1348,7 @@
         <v>2405</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>888</v>
+        <v>892</v>
       </c>
       <c r="E9" s="25" t="inlineStr">
         <is>
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="F9" s="23" t="n">
-        <v>1517</v>
+        <v>1513</v>
       </c>
     </row>
     <row r="10">
@@ -1400,7 +1400,7 @@
         <v>4688</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>1541</v>
+        <v>1554</v>
       </c>
       <c r="E11" s="25" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="F11" s="23" t="n">
-        <v>3147</v>
+        <v>3134</v>
       </c>
     </row>
     <row r="12">
@@ -1423,18 +1423,18 @@
         </is>
       </c>
       <c r="C12" s="23" t="n">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E12" s="25" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>36%</t>
         </is>
       </c>
       <c r="F12" s="23" t="n">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13">
@@ -1452,15 +1452,15 @@
         <v>1530</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>921</v>
+        <v>961</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>63%</t>
         </is>
       </c>
       <c r="F13" s="23" t="n">
-        <v>609</v>
+        <v>569</v>
       </c>
     </row>
     <row r="14">
@@ -1527,10 +1527,10 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>12285</v>
+        <v>12284</v>
       </c>
       <c r="D16" s="27" t="n">
-        <v>3995</v>
+        <v>4057</v>
       </c>
       <c r="E16" s="25" t="inlineStr">
         <is>
@@ -1538,7 +1538,7 @@
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>8290</v>
+        <v>8227</v>
       </c>
     </row>
     <row r="17">
@@ -1582,15 +1582,15 @@
         <v>5888</v>
       </c>
       <c r="D18" s="23" t="n">
-        <v>1850</v>
+        <v>1888</v>
       </c>
       <c r="E18" s="25" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="F18" s="23" t="n">
-        <v>4038</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="19">
@@ -1634,7 +1634,7 @@
         <v>2454</v>
       </c>
       <c r="D20" s="23" t="n">
-        <v>1096</v>
+        <v>1116</v>
       </c>
       <c r="E20" s="25" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
         </is>
       </c>
       <c r="F20" s="23" t="n">
-        <v>1358</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="21">
@@ -1660,15 +1660,15 @@
         <v>553</v>
       </c>
       <c r="D21" s="23" t="n">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="E21" s="26" t="inlineStr">
         <is>
-          <t>51%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="F21" s="23" t="n">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="22">
@@ -1686,15 +1686,15 @@
         <v>1656</v>
       </c>
       <c r="D22" s="23" t="n">
-        <v>1228</v>
+        <v>1248</v>
       </c>
       <c r="E22" s="26" t="inlineStr">
         <is>
-          <t>74%</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="F22" s="23" t="n">
-        <v>428</v>
+        <v>408</v>
       </c>
     </row>
     <row r="23">
@@ -1764,7 +1764,7 @@
         <v>10823</v>
       </c>
       <c r="D25" s="27" t="n">
-        <v>4608</v>
+        <v>4693</v>
       </c>
       <c r="E25" s="25" t="inlineStr">
         <is>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>6215</v>
+        <v>6130</v>
       </c>
     </row>
     <row r="26">
@@ -1868,15 +1868,15 @@
         <v>200</v>
       </c>
       <c r="D29" s="23" t="n">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="E29" s="26" t="inlineStr">
         <is>
-          <t>72%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="F29" s="23" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30">
@@ -1998,15 +1998,15 @@
         <v>397</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="E34" s="25" t="inlineStr">
         <is>
-          <t>47%</t>
+          <t>49%</t>
         </is>
       </c>
       <c r="F34" s="27" t="n">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="35">
@@ -2021,18 +2021,18 @@
         </is>
       </c>
       <c r="C35" s="29" t="n">
-        <v>23533</v>
+        <v>23532</v>
       </c>
       <c r="D35" s="29" t="n">
-        <v>8810</v>
+        <v>8963</v>
       </c>
       <c r="E35" s="25" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="F35" s="29" t="n">
-        <v>14723</v>
+        <v>14569</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
@@ -2171,10 +2171,10 @@
         <v>371</v>
       </c>
       <c r="C42" s="23" t="n">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D42" s="23" t="n">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E42" s="23" t="n">
         <v>358</v>
@@ -2239,19 +2239,19 @@
         <v>70</v>
       </c>
       <c r="C44" s="23" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D44" s="23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E44" s="23" t="n">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="F44" s="23" t="n">
         <v>20</v>
       </c>
       <c r="G44" s="23" t="n">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="H44" s="23" t="n">
         <v>43</v>
@@ -2279,22 +2279,22 @@
         <v>48</v>
       </c>
       <c r="E45" s="23" t="n">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="F45" s="23" t="n">
         <v>50</v>
       </c>
       <c r="G45" s="23" t="n">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="H45" s="23" t="n">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="I45" s="23" t="n">
         <v>79</v>
       </c>
       <c r="J45" s="23" t="n">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="46">
@@ -2313,13 +2313,13 @@
         <v>7</v>
       </c>
       <c r="E46" s="23" t="n">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="F46" s="23" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G46" s="23" t="n">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="H46" s="23" t="n">
         <v>9</v>
@@ -2409,28 +2409,28 @@
         <v>669</v>
       </c>
       <c r="C49" s="29" t="n">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="D49" s="29" t="n">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E49" s="29" t="n">
-        <v>1530</v>
+        <v>1554</v>
       </c>
       <c r="F49" s="29" t="n">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G49" s="29" t="n">
-        <v>1187</v>
+        <v>1210</v>
       </c>
       <c r="H49" s="29" t="n">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="I49" s="29" t="n">
         <v>106</v>
       </c>
       <c r="J49" s="29" t="n">
-        <v>415</v>
+        <v>418</v>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">

</xml_diff>

<commit_message>
FIX erase/edit race: PEND lock protects just-committed local edits from 1.1s pull reverting them before 400ms push fires (LIVE v6)
</commit_message>
<xml_diff>
--- a/EXCEL/1 - DASHBOARD.xlsx
+++ b/EXCEL/1 - DASHBOARD.xlsx
@@ -65,7 +65,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FFc00000"/>
+      <color rgb="FFed7d31"/>
       <sz val="10"/>
     </font>
     <font>
@@ -77,7 +77,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FFed7d31"/>
+      <color rgb="FFc00000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -672,9 +672,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -684,10 +681,13 @@
     <xf numFmtId="0" fontId="10" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="25" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -699,7 +699,7 @@
     <xf numFmtId="0" fontId="5" fillId="27" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1147,11 +1147,11 @@
         <v>23532</v>
       </c>
       <c r="B2" s="9" t="n">
-        <v>8963</v>
+        <v>9092</v>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="D2" s="11" t="n">
@@ -1167,7 +1167,7 @@
         <v>290</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
@@ -1348,7 +1348,7 @@
         <v>2405</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>892</v>
+        <v>894</v>
       </c>
       <c r="E9" s="25" t="inlineStr">
         <is>
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="F9" s="23" t="n">
-        <v>1513</v>
+        <v>1511</v>
       </c>
     </row>
     <row r="10">
@@ -1400,15 +1400,15 @@
         <v>4688</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>1554</v>
+        <v>1587</v>
       </c>
       <c r="E11" s="25" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="F11" s="23" t="n">
-        <v>3134</v>
+        <v>3101</v>
       </c>
     </row>
     <row r="12">
@@ -1452,7 +1452,7 @@
         <v>1530</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>961</v>
+        <v>964</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="F13" s="23" t="n">
-        <v>569</v>
+        <v>566</v>
       </c>
     </row>
     <row r="14">
@@ -1530,7 +1530,7 @@
         <v>12284</v>
       </c>
       <c r="D16" s="27" t="n">
-        <v>4057</v>
+        <v>4095</v>
       </c>
       <c r="E16" s="25" t="inlineStr">
         <is>
@@ -1538,7 +1538,7 @@
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>8227</v>
+        <v>8189</v>
       </c>
     </row>
     <row r="17">
@@ -1582,15 +1582,15 @@
         <v>5888</v>
       </c>
       <c r="D18" s="23" t="n">
-        <v>1888</v>
+        <v>1947</v>
       </c>
       <c r="E18" s="25" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="F18" s="23" t="n">
-        <v>4000</v>
+        <v>3941</v>
       </c>
     </row>
     <row r="19">
@@ -1634,15 +1634,15 @@
         <v>2454</v>
       </c>
       <c r="D20" s="23" t="n">
-        <v>1116</v>
+        <v>1133</v>
       </c>
       <c r="E20" s="25" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>46%</t>
         </is>
       </c>
       <c r="F20" s="23" t="n">
-        <v>1338</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="21">
@@ -1686,15 +1686,15 @@
         <v>1656</v>
       </c>
       <c r="D22" s="23" t="n">
-        <v>1248</v>
+        <v>1263</v>
       </c>
       <c r="E22" s="26" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="F22" s="23" t="n">
-        <v>408</v>
+        <v>393</v>
       </c>
     </row>
     <row r="23">
@@ -1764,15 +1764,15 @@
         <v>10823</v>
       </c>
       <c r="D25" s="27" t="n">
-        <v>4693</v>
+        <v>4784</v>
       </c>
       <c r="E25" s="25" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>44%</t>
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>6130</v>
+        <v>6039</v>
       </c>
     </row>
     <row r="26">
@@ -2024,15 +2024,15 @@
         <v>23532</v>
       </c>
       <c r="D35" s="29" t="n">
-        <v>8963</v>
+        <v>9092</v>
       </c>
       <c r="E35" s="25" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="F35" s="29" t="n">
-        <v>14569</v>
+        <v>14440</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">

</xml_diff>